<commit_message>
test: add ReqRes pagination test
</commit_message>
<xml_diff>
--- a/JuiceShop test-cases.xlsx
+++ b/JuiceShop test-cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\INNOWISE\AQA intern\AQA\ДЗ №5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\INNOWISE\AQA intern\AQA\JS-automation-basics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{312AAB01-BE88-4519-A9A5-19D1DEB72503}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB8087A4-2D03-4400-8A29-75A900FFB82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="324">
   <si>
     <t>ID</t>
   </si>
@@ -1425,9 +1425,6 @@
   </si>
   <si>
     <t>executed in fixtures/api.js with status check</t>
-  </si>
-  <si>
-    <t>Postman</t>
   </si>
 </sst>
 </file>
@@ -2641,9 +2638,7 @@
       <c r="G3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H3" s="14"/>
     </row>
     <row r="4" spans="1:8" ht="71.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
@@ -2667,9 +2662,7 @@
       <c r="G4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H4" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H4" s="14"/>
     </row>
     <row r="5" spans="1:8" ht="71.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
@@ -2693,9 +2686,7 @@
       <c r="G5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H5" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H5" s="14"/>
     </row>
     <row r="6" spans="1:8" ht="84.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
@@ -2719,9 +2710,7 @@
       <c r="G6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H6" s="14"/>
     </row>
     <row r="7" spans="1:8" ht="71.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
@@ -2745,9 +2734,7 @@
       <c r="G7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H7" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H7" s="14"/>
     </row>
     <row r="8" spans="1:8" ht="59" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
@@ -2771,9 +2758,7 @@
       <c r="G8" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H8" s="14"/>
     </row>
     <row r="9" spans="1:8" ht="71.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
@@ -2797,9 +2782,7 @@
       <c r="G9" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H9" s="14"/>
     </row>
     <row r="10" spans="1:8" ht="71.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
@@ -3031,9 +3014,7 @@
       <c r="G18" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="H18" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H18" s="14"/>
     </row>
     <row r="19" spans="1:8" ht="84.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="4" t="s">
@@ -3057,9 +3038,7 @@
       <c r="G19" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H19" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H19" s="14"/>
     </row>
     <row r="20" spans="1:8" ht="71.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="4" t="s">
@@ -3083,9 +3062,7 @@
       <c r="G20" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H20" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H20" s="14"/>
     </row>
     <row r="21" spans="1:8" ht="59" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
@@ -3109,9 +3086,7 @@
       <c r="G21" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H21" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H21" s="14"/>
     </row>
     <row r="22" spans="1:8" ht="71.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4" t="s">
@@ -3135,9 +3110,7 @@
       <c r="G22" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H22" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H22" s="14"/>
     </row>
     <row r="23" spans="1:8" ht="71.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="4" t="s">
@@ -3161,9 +3134,7 @@
       <c r="G23" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H23" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H23" s="14"/>
     </row>
     <row r="24" spans="1:8" ht="84.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="4" t="s">
@@ -3187,9 +3158,7 @@
       <c r="G24" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H24" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H24" s="14"/>
     </row>
     <row r="25" spans="1:8" ht="59" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="4" t="s">
@@ -3213,9 +3182,7 @@
       <c r="G25" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H25" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H25" s="14"/>
     </row>
     <row r="26" spans="1:8" ht="84.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="4" t="s">
@@ -3239,9 +3206,7 @@
       <c r="G26" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H26" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H26" s="14"/>
     </row>
     <row r="27" spans="1:8" ht="84.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="4" t="s">
@@ -3265,9 +3230,7 @@
       <c r="G27" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H27" s="14" t="s">
-        <v>324</v>
-      </c>
+      <c r="H27" s="14"/>
     </row>
     <row r="28" spans="1:8" ht="71.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="4" t="s">

</xml_diff>